<commit_message>
fix(feed): BACI 490 "Other Asia, nes" maps to Taiwan instead of ROW, and the netting refuses a source version whose region map differs from current's — Taiwan gains trade, ROW loses Taiwan's 375–655 kt/yr of cathode imports; measured by #79 (ADR 0014, 0018 am., #77)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/feed/baci/current/conc.xlsx
+++ b/data/input/feed/baci/current/conc.xlsx
@@ -889,7 +889,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -910,7 +909,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1081,7 +1079,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1102,7 +1099,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1298,7 +1294,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1369,7 +1364,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1415,7 +1409,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1586,7 +1579,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1682,7 +1674,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1703,7 +1694,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1724,7 +1714,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1745,7 +1734,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2116,7 +2104,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -2512,7 +2499,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -2608,7 +2594,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -2754,7 +2739,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -2825,7 +2809,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -3121,7 +3104,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -3142,7 +3124,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -3163,7 +3144,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -3259,7 +3239,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -3305,7 +3284,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -3351,7 +3329,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -3647,7 +3624,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -3718,7 +3694,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -3839,7 +3814,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -3910,7 +3884,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -3931,7 +3904,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -4177,7 +4149,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -4198,7 +4169,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -4456,12 +4426,12 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>ROW</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>aggregate</t>
+          <t>alias</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -4471,7 +4441,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>Corrected from 'RoW'</t>
+          <t>'Other Asia, nes' is Taiwan's trade in UN Comtrade and BACI; was ROW (#77)</t>
         </is>
       </c>
     </row>
@@ -4544,7 +4514,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -4565,7 +4534,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -4611,7 +4579,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -4632,7 +4599,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -4678,7 +4644,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -4699,7 +4664,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -5270,7 +5234,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -5291,7 +5254,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -5387,7 +5349,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -5458,7 +5419,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -5604,7 +5564,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -5625,7 +5584,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -6021,7 +5979,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -6042,7 +5999,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -6188,7 +6144,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -6334,7 +6289,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -7052,7 +7006,6 @@
           <t>src_time</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>cast to str → time_map</t>
@@ -7080,7 +7033,6 @@
           <t>src_sector_from</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>direct → sector_map (HS code)</t>
@@ -7108,7 +7060,6 @@
           <t>src_region_from</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>direct → region_map (numeric ID)</t>
@@ -7136,7 +7087,6 @@
           <t>src_region_to</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>direct → region_map (numeric ID)</t>
@@ -7164,7 +7114,6 @@
           <t>src_valuation</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>direct → valuation_map</t>

</xml_diff>

<commit_message>
fix(feed): the 490 row is typed direct with its ICSG provenance, a test maps a 490 row through the registered region map, the ADRs leave the numbers to #79, and the glossary defines observation instead of narrating it (review of 40f3ac4, #77)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/feed/baci/current/conc.xlsx
+++ b/data/input/feed/baci/current/conc.xlsx
@@ -4431,7 +4431,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>alias</t>
+          <t>direct</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -4441,7 +4441,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>'Other Asia, nes' is Taiwan's trade in UN Comtrade and BACI; was ROW (#77)</t>
+          <t>'Other Asia, nes' is Taiwan's trade in UN Comtrade and BACI; its cathode imports track ICSG's Taiwan usage (#77); was ROW</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(feed): BACI 178 "Congo" maps to Congo, D.R. and 711 "Southern African Customs Union" to South Africa — ROW no longer exports 3,890 kt of DR Congo's cathode in 2012–2024 nor carries South Africa's 1995–1999 trade (ADR 0014 am., #84)
178 exported 3,890 kt of cathode (HS 740311) in 2012–2024, mostly to the UAE, Italy and Greece, against
Brazzaville's 79 kt of ICSG production and DR Congo's 2,752 kt CC shortfall under 180. 711 is South
Africa's trade, with Namibia's and Botswana's, until BACI splits it in 2000. Both rows are `direct`, as
490 → Taiwan (#77). Neither creates mapped self-trade: BACI has no 178 ↔ 180 or 711 ↔ 710 rows. South
Africa and DR Congo were already BACI-observed (any year), so ADR 0018's set is unchanged.

The map is the unregistered current/conc.xlsx; #86 registers and measures it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/feed/baci/current/conc.xlsx
+++ b/data/input/feed/baci/current/conc.xlsx
@@ -1841,12 +1841,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ROW</t>
+          <t>Congo, D.R.</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>aggregate</t>
+          <t>direct</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Corrected from 'RoW'</t>
+          <t>BACI's 'Congo' carries DR Congo's cathode: 3,890 kt exported in 2012–2024 against Brazzaville's 79 kt of ICSG production and DR Congo's shortfall under 180 (#84); was ROW</t>
         </is>
       </c>
     </row>
@@ -5381,12 +5381,12 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>ROW</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>aggregate</t>
+          <t>direct</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -5396,7 +5396,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>Corrected from 'RoW'</t>
+          <t>'Southern African Customs Union' is South Africa's trade until BACI splits it in 2000; Namibia's anode and Botswana's matte ride with it (#84); was ROW</t>
         </is>
       </c>
     </row>

</xml_diff>